<commit_message>
Import template: optional fault date column so historical data keeps its real dates
</commit_message>
<xml_diff>
--- a/samples/maintrack-import-demo.xlsx
+++ b/samples/maintrack-import-demo.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -49,9 +52,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -429,6 +433,7 @@
     <col width="25" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
     <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,6 +482,11 @@
           <t>Χρόνος Διακοπής (λεπτά)</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Ημερομηνία Βλάβης</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -522,6 +532,9 @@
       <c r="I2" t="n">
         <v>90</v>
       </c>
+      <c r="J2" s="2" t="n">
+        <v>46125</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -567,6 +580,9 @@
       <c r="I3" t="n">
         <v>50</v>
       </c>
+      <c r="J3" s="2" t="n">
+        <v>46147</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -604,8 +620,9 @@
           <t>d.georgiou</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
+        <v>46172</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -651,6 +668,9 @@
       <c r="I5" t="n">
         <v>30</v>
       </c>
+      <c r="J5" s="2" t="n">
+        <v>46189</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -683,7 +703,6 @@
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Καθαρισμός και προστασία μπάρας</t>
@@ -692,6 +711,9 @@
       <c r="I6" t="n">
         <v>25</v>
       </c>
+      <c r="J6" s="2" t="n">
+        <v>46210</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -724,9 +746,9 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
+        <v>46223</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -759,9 +781,9 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
+        <v>46223</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -799,8 +821,9 @@
           <t>a.anyparktos</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>46223</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -813,7 +836,6 @@
           <t>FUR2</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>Λείπει ο τίτλος της βλάβης</t>
@@ -829,9 +851,9 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
+        <v>46223</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -876,6 +898,9 @@
       </c>
       <c r="I11" t="n">
         <v>90</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>46125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>